<commit_message>
feat(pedagogia): adicionar secao Follow-up com educativos e calibrar tom sem superlativos
</commit_message>
<xml_diff>
--- a/PRONTUARIO_E_HISTORICO_GUILHERME_LEMOS.xlsx
+++ b/PRONTUARIO_E_HISTORICO_GUILHERME_LEMOS.xlsx
@@ -1433,7 +1433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1444,7 +1444,8 @@
     <col width="38" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1497,11 +1498,16 @@
       </c>
       <c r="I2" s="22" t="inlineStr">
         <is>
+          <t>Follow-up (Ajustes &amp; Educativos)</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="44" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>02/10/2026</t>
@@ -1534,21 +1540,26 @@
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>Subida suave sem salto flutuando o quadril sobre a base. Alinhamento perpendicular impecável e descida macia.</t>
+          <t>O parceiro de baixo mantém joelhos semifletidos para estabilidade. O Gui apoia nos ombros dele, projeta o tronco à frente e sobe o quadril sem salto. No topo, abre em straddle mantendo o alinhamento sobre a coluna da base e desce suavemente.</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>Empilhamento ósseo (bone stacking). Translação escapular projeta centro de gravidade sobre clavículas da base; desaceleração por peitoral menor.</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
+          <t>Empilhamento ósseo com absorção da carga axial (~84 kg) pela base; translação escapular que projeta o centro de gravidade sobre as clavículas; desaceleração excêntrica conduzida por peitoral menor e trapézio inferior.</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Ajuste fino: reduzir sutilmente a anteversão pélvica na abertura das pernas. Educativo: press to handstand com apoio na parede na paralela baixa (3x3 com pausa de 3s). Próximo passo: subida com pernas unidas (pike press).</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>02/10/2026</t>
@@ -1581,21 +1592,26 @@
       </c>
       <c r="G4" s="19" t="inlineStr">
         <is>
-          <t>Retorno triunfal após 2 anos preservando o ombro. False grip firme, passagem de cotovelos colados e subida em vela fluída.</t>
+          <t>Retorno às argolas com subida estrita. Pegada falsa com punho flexionado, puxada até o peito na altura das mãos e cotovelos colados sem impulso de pernas. Em seguida, descida em vela e balanço com braços esticados para retornar ao apoio.</t>
         </is>
       </c>
       <c r="H4" s="19" t="inlineStr">
         <is>
-          <t>Flexão ulnocarpal elimina braço de alavanca parasita; adução de ombro rente às costelas e conversão de energia angular no candle kip.</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
+          <t>Flexão ulnocarpal profunda elimina defasagem mecânica do punho, poupando a articulação glenoumeral no ombro operado e inserção do tríceps; candle kip converte energia potencial em momento angular por tração estendida.</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Ajuste fino: manter pernas e pontas dos pés ativas na transição do dip. Educativo: transições lentas na argola baixa com pés no solo (3x5 reps). Próximo passo: séries de 2 a 3 repetições estritas consecutivas.</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>01/10/2026</t>
@@ -1628,21 +1644,26 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>Início em L-sit, subida lenta em straddle press sem embalo, trava perfeita de 10s e One-Arm Croc cravado por 7 segundos.</t>
+          <t>Entrada em L-sit estático suspenso, subida contínua sem embalo até a parada de mãos aberta, trava estável por 8s, descida controlada e encaixe do cotovelo na bacia para One-Arm Crocodile por 7s com o outro braço estendido.</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>Fulcro no olécrano e espinha ilíaca ântero-superior; torque rotacional severo contra a gravidade sustentado por oblíquos contralaterais.</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
+          <t>Força concêntrica de flexores de quadril e deltóide anterior com elevação escapular mantida; apoio do olécrano na espinha ilíaca ântero-superior e torque anti-rotacional neutralizado por oblíquos contralaterais.</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Ajuste fino: nivelar o tronco paralelamente ao solo no Crocodile. Educativo: isometria na manjota com apoio de 2 dedos da mão livre (3x 8-10s por lado). Próximo passo: transição de volta para duas mãos sem tocar o solo.</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>01/10/2026</t>
@@ -1675,21 +1696,26 @@
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
-          <t>Balanço elástico rente ao solo, fechamento pélvico colando pés na barra e elevação em bloqueio ósseo com troca rápida de punhos.</t>
+          <t>Balanço amplo perto do chão, flexão de quadril aproximando as canelas da barra no retorno do pêndulo e puxada com cotovelos estendidos até o apoio sobre a barra, encadeando 4 repetições contínuas com ritmo constante.</t>
         </is>
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>Extensão pura de ombro com grande dorsal e tríceps longo; timing na reversão do pêndulo angular da ginástica artística.</t>
-        </is>
-      </c>
-      <c r="I6" s="13" t="inlineStr">
+          <t>Timing na reversão do pêndulo angular encurtando o raio de rotação para ascensão vertical; extensão de ombro com grande dorsal e tríceps cabeça longa com rápida troca de punhos por cima do eixo.</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Ajuste fino: abrir o peito na subida ao apoio para entrar com os ombros projetados à frente. Educativo: balanço de oitava com bola medicinal leve entre tornozelos (3x6 reps). Próximo passo: saída da oitava ligada em giro para trás.</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7" ht="44" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>05/10/2026</t>
@@ -1722,15 +1748,20 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>Perda visível de gordura abdominal e preservação de tônus muscular, confirmando -13kg de massa gorda sem atrofia.</t>
+          <t>Comparativo fotográfico evidenciando redução da adiposidade abdominal e definição do contorno muscular em 95 dias de acompanhamento, com preservação da estrutura muscular em tronco e braços.</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>Descompressão de 40-50kg no platô tibial por ciclo de passo/agachamento; aumento expressivo de W/kg.</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr">
+          <t>Estímulo tensional frequente e aporte proteico de 2.0 a 2.4 g/kg preservando massa magra; descompressão de 40 a 50 kg no platô tibial por ciclo de passo/agachamento (-13 kg acumulados).</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Ajuste fino: manter taxa de perda controlada (~0.8 a 1.0 kg/sem) com bioimpedância mensal. Conduta sugerida: refeed limpo sincronizado com treinos de alta densidade. Próximo passo: consolidação em 80-82 kg com 14% de gordura.</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
@@ -1738,7 +1769,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(pedagogia): inverter botoes para Analises antes de Evolucao e dividir em Diagnostico e Exercicios Sugeridos
</commit_message>
<xml_diff>
--- a/PRONTUARIO_E_HISTORICO_GUILHERME_LEMOS.xlsx
+++ b/PRONTUARIO_E_HISTORICO_GUILHERME_LEMOS.xlsx
@@ -1433,19 +1433,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1498,16 +1499,21 @@
       </c>
       <c r="I2" s="22" t="inlineStr">
         <is>
-          <t>Follow-up (Ajustes &amp; Educativos)</t>
+          <t>Diagnóstico (O que ajustar)</t>
         </is>
       </c>
       <c r="J2" s="22" t="inlineStr">
         <is>
+          <t>Exercícios Sugeridos</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="44" customHeight="1">
+    <row r="3" ht="46" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>02/10/2026</t>
@@ -1550,16 +1556,22 @@
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>Ajuste fino: reduzir sutilmente a anteversão pélvica na abertura das pernas. Educativo: press to handstand com apoio na parede na paralela baixa (3x3 com pausa de 3s). Próximo passo: subida com pernas unidas (pike press).</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
+          <t>A subida foi muito suave e estável. No topo, ao abrir as pernas, o quadril empina um pouco para trás e a lombar curva de leve. Basta travar bem a barriga e o bumbum para a coluna subir reta.</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>• Press na paralela baixa com costas na parede (3x3 com pausa de 3s no topo).
+• Subida no ombro com pernas unidas (pike press) para ganhar mais força de compressão.</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
+    <row r="4" ht="46" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
           <t>02/10/2026</t>
@@ -1602,16 +1614,22 @@
       </c>
       <c r="I4" s="19" t="inlineStr">
         <is>
-          <t>Ajuste fino: manter pernas e pontas dos pés ativas na transição do dip. Educativo: transições lentas na argola baixa com pés no solo (3x5 reps). Próximo passo: séries de 2 a 3 repetições estritas consecutivas.</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
+          <t>Subida de força muito segura para o ombro operado. Na passagem para empurrar o apoio, os joelhos deram uma leve dobrada. As pernas devem ficar 100% esticadas e pontas dos pés ativas.</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>• Transições lentas na argola baixa com pés no chão (3x5 reps com cotovelos colados).
+• Séries de 2 a 3 repetições estritas consecutivas mantendo a pegada falsa firme.</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
+    <row r="5" ht="46" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>01/10/2026</t>
@@ -1654,16 +1672,22 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>Ajuste fino: nivelar o tronco paralelamente ao solo no Crocodile. Educativo: isometria na manjota com apoio de 2 dedos da mão livre (3x 8-10s por lado). Próximo passo: transição de volta para duas mãos sem tocar o solo.</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
+          <t>L-sit e subida na parada de mãos impecáveis. No apoio de um braço só (Crocodile), o quadril deu uma leve caída para o lado. O corpo precisa ficar reto como uma prancha paralela ao chão.</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>• Isometria na manjota com apoio de apenas 2 dedos da mão livre (3x 8-10s por lado).
+• Retorno do Crocodile para as duas mãos sem encostar os pés no chão.</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1">
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>01/10/2026</t>
@@ -1706,16 +1730,22 @@
       </c>
       <c r="I6" s="19" t="inlineStr">
         <is>
-          <t>Ajuste fino: abrir o peito na subida ao apoio para entrar com os ombros projetados à frente. Educativo: balanço de oitava com bola medicinal leve entre tornozelos (3x6 reps). Próximo passo: saída da oitava ligada em giro para trás.</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="inlineStr">
+          <t>Excelente ritmo nas 4 repetições. Na subida em cima da barra, o peito ainda sobe um pouco recolhido. Abra o peito e projete os ombros à frente da barra para embalar fácil na repetição seguinte.</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>• Balanço de oitava segurando bola medicinal leve entre os tornozelos (3x6 reps).
+• Saída da oitava ligada direto no giro de apoio para trás na barra.</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="44" customHeight="1">
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>05/10/2026</t>
@@ -1758,10 +1788,16 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Ajuste fino: manter taxa de perda controlada (~0.8 a 1.0 kg/sem) com bioimpedância mensal. Conduta sugerida: refeed limpo sincronizado com treinos de alta densidade. Próximo passo: consolidação em 80-82 kg com 14% de gordura.</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
+          <t>Perda de peso consistente e com ótima retenção de massa muscular. Manter a disciplina para não acelerar demais e garantir a preservação da força nas habilidades gímnicas.</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>• Manter ingestão proteica alta (2.0-2.4 g/kg) e hidratação rigorosa.
+• Refeed limpo sincronizado com dias de treinos mais pesados na EEFERP.</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
         </is>
@@ -1769,7 +1805,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(pedagogia): padronizar 4 blocos nas analises de video e simplificar instrucoes regulares
</commit_message>
<xml_diff>
--- a/PRONTUARIO_E_HISTORICO_GUILHERME_LEMOS.xlsx
+++ b/PRONTUARIO_E_HISTORICO_GUILHERME_LEMOS.xlsx
@@ -1494,17 +1494,17 @@
       </c>
       <c r="H2" s="22" t="inlineStr">
         <is>
+          <t>Diagnóstico (O que ajustar)</t>
+        </is>
+      </c>
+      <c r="I2" s="22" t="inlineStr">
+        <is>
+          <t>Exercícios Sugeridos</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
           <t>Base Científica &amp; Origem</t>
-        </is>
-      </c>
-      <c r="I2" s="22" t="inlineStr">
-        <is>
-          <t>Diagnóstico (O que ajustar)</t>
-        </is>
-      </c>
-      <c r="J2" s="22" t="inlineStr">
-        <is>
-          <t>Exercícios Sugeridos</t>
         </is>
       </c>
       <c r="K2" s="22" t="inlineStr">
@@ -1551,20 +1551,20 @@
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>Empilhamento ósseo com absorção da carga axial (~84 kg) pela base; translação escapular que projeta o centro de gravidade sobre as clavículas; desaceleração excêntrica conduzida por peitoral menor e trapézio inferior.</t>
+          <t>A subida foi muito suave e estável. No topo, ao abrir as pernas, o quadril empina um pouco para trás e a lombar curva de leve. Basta travar bem a barriga e o bumbum para a coluna subir reta.</t>
         </is>
       </c>
       <c r="I3" s="15" t="inlineStr">
-        <is>
-          <t>A subida foi muito suave e estável. No topo, ao abrir as pernas, o quadril empina um pouco para trás e a lombar curva de leve. Basta travar bem a barriga e o bumbum para a coluna subir reta.</t>
-        </is>
-      </c>
-      <c r="J3" s="15" t="inlineStr">
         <is>
           <t>• Press na paralela baixa com costas na parede (3x3 com pausa de 3s no topo).
 • Subida no ombro com pernas unidas (pike press) para ganhar mais força de compressão.</t>
         </is>
       </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Empilhamento ósseo com absorção da carga axial (~84 kg) pela base; translação escapular que projeta o centro de gravidade sobre as clavículas; desaceleração excêntrica conduzida por peitoral menor e trapézio inferior.</t>
+        </is>
+      </c>
       <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
@@ -1609,20 +1609,20 @@
       </c>
       <c r="H4" s="19" t="inlineStr">
         <is>
-          <t>Flexão ulnocarpal profunda elimina defasagem mecânica do punho, poupando a articulação glenoumeral no ombro operado e inserção do tríceps; candle kip converte energia potencial em momento angular por tração estendida.</t>
+          <t>Subida de força muito segura para o ombro operado. Na passagem para empurrar o apoio, os joelhos deram uma leve dobrada. As pernas devem ficar 100% esticadas e pontas dos pés ativas.</t>
         </is>
       </c>
       <c r="I4" s="19" t="inlineStr">
-        <is>
-          <t>Subida de força muito segura para o ombro operado. Na passagem para empurrar o apoio, os joelhos deram uma leve dobrada. As pernas devem ficar 100% esticadas e pontas dos pés ativas.</t>
-        </is>
-      </c>
-      <c r="J4" s="19" t="inlineStr">
         <is>
           <t>• Transições lentas na argola baixa com pés no chão (3x5 reps com cotovelos colados).
 • Séries de 2 a 3 repetições estritas consecutivas mantendo a pegada falsa firme.</t>
         </is>
       </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>Flexão ulnocarpal profunda elimina defasagem mecânica do punho, poupando a articulação glenoumeral no ombro operado e inserção do tríceps; candle kip converte energia potencial em momento angular por tração estendida.</t>
+        </is>
+      </c>
       <c r="K4" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
@@ -1667,20 +1667,20 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>Força concêntrica de flexores de quadril e deltóide anterior com elevação escapular mantida; apoio do olécrano na espinha ilíaca ântero-superior e torque anti-rotacional neutralizado por oblíquos contralaterais.</t>
+          <t>L-sit e subida na parada de mãos impecáveis. No apoio de um braço só (Crocodile), o quadril deu uma leve caída para o lado. O corpo precisa ficar reto como uma prancha paralela ao chão.</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>L-sit e subida na parada de mãos impecáveis. No apoio de um braço só (Crocodile), o quadril deu uma leve caída para o lado. O corpo precisa ficar reto como uma prancha paralela ao chão.</t>
-        </is>
-      </c>
-      <c r="J5" s="15" t="inlineStr">
         <is>
           <t>• Isometria na manjota com apoio de apenas 2 dedos da mão livre (3x 8-10s por lado).
 • Retorno do Crocodile para as duas mãos sem encostar os pés no chão.</t>
         </is>
       </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Força concêntrica de flexores de quadril e deltóide anterior com elevação escapular mantida; apoio do olécrano na espinha ilíaca ântero-superior e torque anti-rotacional neutralizado por oblíquos contralaterais.</t>
+        </is>
+      </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
@@ -1725,20 +1725,20 @@
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>Timing na reversão do pêndulo angular encurtando o raio de rotação para ascensão vertical; extensão de ombro com grande dorsal e tríceps cabeça longa com rápida troca de punhos por cima do eixo.</t>
+          <t>Excelente ritmo nas 4 repetições. Na subida em cima da barra, o peito ainda sobe um pouco recolhido. Abra o peito e projete os ombros à frente da barra para embalar fácil na repetição seguinte.</t>
         </is>
       </c>
       <c r="I6" s="19" t="inlineStr">
-        <is>
-          <t>Excelente ritmo nas 4 repetições. Na subida em cima da barra, o peito ainda sobe um pouco recolhido. Abra o peito e projete os ombros à frente da barra para embalar fácil na repetição seguinte.</t>
-        </is>
-      </c>
-      <c r="J6" s="19" t="inlineStr">
         <is>
           <t>• Balanço de oitava segurando bola medicinal leve entre os tornozelos (3x6 reps).
 • Saída da oitava ligada direto no giro de apoio para trás na barra.</t>
         </is>
       </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>Timing na reversão do pêndulo angular encurtando o raio de rotação para ascensão vertical; extensão de ombro com grande dorsal e tríceps cabeça longa com rápida troca de punhos por cima do eixo.</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
           <t>Validado ✅</t>
@@ -1783,18 +1783,18 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>Estímulo tensional frequente e aporte proteico de 2.0 a 2.4 g/kg preservando massa magra; descompressão de 40 a 50 kg no platô tibial por ciclo de passo/agachamento (-13 kg acumulados).</t>
+          <t>Perda de peso consistente e com ótima retenção de massa muscular. Manter a disciplina para não acelerar demais e garantir a preservação da força nas habilidades gímnicas.</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>Perda de peso consistente e com ótima retenção de massa muscular. Manter a disciplina para não acelerar demais e garantir a preservação da força nas habilidades gímnicas.</t>
-        </is>
-      </c>
-      <c r="J7" s="15" t="inlineStr">
         <is>
           <t>• Manter ingestão proteica alta (2.0-2.4 g/kg) e hidratação rigorosa.
 • Refeed limpo sincronizado com dias de treinos mais pesados na EEFERP.</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>Estímulo tensional frequente e aporte proteico de 2.0 a 2.4 g/kg preservando massa magra; descompressão de 40 a 50 kg no platô tibial por ciclo de passo/agachamento (-13 kg acumulados).</t>
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr">

</xml_diff>